<commit_message>
added transformer and gap pad drawing
</commit_message>
<xml_diff>
--- a/bom/OSLUV_Excimer-Driver.xlsx
+++ b/bom/OSLUV_Excimer-Driver.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Unsere_Geräte\Ushio Care222\OSLUV\06_Produktion\Stücklisten\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Unsere_Geräte\Ushio Care222\OSLUV\09_Zeichnungen\Zeichnungen\KiCAD\OSLUV\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA0D826C-49D7-4238-9517-49C5354BD25A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EBB302B-A3F1-4FB3-8543-806B399ABB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{68E81C6F-E3AF-44B4-92E9-C765077DD5C1}"/>
+    <workbookView xWindow="5715" yWindow="2655" windowWidth="21600" windowHeight="11280" xr2:uid="{68E81C6F-E3AF-44B4-92E9-C765077DD5C1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -533,9 +533,6 @@
     <t>M2</t>
   </si>
   <si>
-    <t>Gap Pad für T101</t>
-  </si>
-  <si>
     <t>MLZ2012N100LT000</t>
   </si>
   <si>
@@ -554,9 +551,6 @@
     <t>ETD29 Celinius</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>ERJ8CWFR020V</t>
   </si>
   <si>
@@ -597,13 +591,40 @@
   </si>
   <si>
     <t>SiC MOFEST 1200V/78mOhm, TO247-4</t>
+  </si>
+  <si>
+    <t>Gap Pad for T101</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Silicone gap pad, 200µm, Ubd≥5kV, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+      </rPr>
+      <t>λ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>≥1.9 W/mK. 24 x 22 mm. Acc. to drawing from 08.01.2026</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -618,6 +639,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -983,7 +1010,7 @@
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="84" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="56.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -998,7 +1025,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -1015,7 +1042,7 @@
         <v>150</v>
       </c>
       <c r="D3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
@@ -1037,7 +1064,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B5">
         <v>12</v>
@@ -1119,7 +1146,7 @@
         <v>155</v>
       </c>
       <c r="D10" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E10" t="s">
         <v>123</v>
@@ -1136,7 +1163,7 @@
         <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E11" t="s">
         <v>17</v>
@@ -1192,7 +1219,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D16" t="s">
         <v>158</v>
@@ -1209,7 +1236,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D18" t="s">
         <v>26</v>
@@ -1282,7 +1309,7 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D24" t="s">
         <v>159</v>
@@ -1299,7 +1326,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="D25" t="s">
         <v>160</v>
@@ -1487,7 +1514,7 @@
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>161</v>
@@ -1504,10 +1531,10 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D42" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E42" t="s">
         <v>73</v>
@@ -1521,7 +1548,7 @@
         <v>2</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E43" t="s">
         <v>74</v>
@@ -1535,7 +1562,7 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D45" t="s">
         <v>163</v>
@@ -1560,10 +1587,10 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="D48" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -1647,7 +1674,7 @@
         <v>84</v>
       </c>
       <c r="D55" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E55" t="s">
         <v>85</v>
@@ -1818,7 +1845,7 @@
         <v>146</v>
       </c>
       <c r="D67" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E67" t="s">
         <v>85</v>
@@ -1846,10 +1873,10 @@
         <v>2</v>
       </c>
       <c r="C69" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D69" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E69" t="s">
         <v>85</v>
@@ -1908,7 +1935,7 @@
         <v>117</v>
       </c>
       <c r="D73" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E73" t="s">
         <v>88</v>
@@ -1964,7 +1991,7 @@
         <v>1</v>
       </c>
       <c r="C79" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D79" t="s">
         <v>156</v>
@@ -1975,5 +2002,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>